<commit_message>
phòng ban, hiệu chỉnh excel in, hiệu chỉnh phiếu chấm công
</commit_message>
<xml_diff>
--- a/ExcelData/UpdateRFID.xlsx
+++ b/ExcelData/UpdateRFID.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\KMALearn\RFID_Project\ExcelData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF5185A4-9C11-4012-8CBC-22F5AEEE0FAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2750A9B8-45F7-4AF3-A217-AF003A33ECDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,10 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
-  <si>
-    <t>Mã sinh viên</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Họ và tên</t>
   </si>
@@ -52,19 +49,34 @@
   </si>
   <si>
     <t>123123451bsdfsdf</t>
+  </si>
+  <si>
+    <t>Mã phòng ban</t>
+  </si>
+  <si>
+    <t>Mã nhân viên</t>
+  </si>
+  <si>
+    <t>sdfsd</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -87,11 +99,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -372,45 +385,55 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.85546875" customWidth="1"/>
     <col min="2" max="2" width="34.140625" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
+    <col min="4" max="4" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
+      <c r="B2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2">
+        <v>123</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>6</v>
       </c>
-      <c r="C3" t="s">
-        <v>7</v>
+      <c r="D3" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>